<commit_message>
Simplify task 1 script and inputs
</commit_message>
<xml_diff>
--- a/task1-bzie0068-covenant-test/upload/inputs/Kestrel_Ridge_Q3_2026_Financials.xlsx
+++ b/task1-bzie0068-covenant-test/upload/inputs/Kestrel_Ridge_Q3_2026_Financials.xlsx
@@ -777,7 +777,6 @@
       <c r="B20" t="n">
         <v>5</v>
       </c>
-      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1522,7 +1521,9 @@
       <c r="B25" s="10" t="n">
         <v>5.25</v>
       </c>
-      <c r="C25" s="11" t="n"/>
+      <c r="C25" s="10" t="n">
+        <v>5.25</v>
+      </c>
       <c r="D25" s="10">
         <f>IF(C25="","",C25-B25)</f>
         <v/>
@@ -1675,15 +1676,14 @@
         </is>
       </c>
       <c r="B38" s="3" t="n"/>
-      <c r="C38" s="7" t="n"/>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="D38" s="3" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Yes,No"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>